<commit_message>
Refa actualizarea produselor din registru
</commit_message>
<xml_diff>
--- a/registru-produse-kymco.xlsx
+++ b/registru-produse-kymco.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4471" uniqueCount="2506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4472" uniqueCount="2507">
   <si>
     <t xml:space="preserve">Cod - Referinta Prestashop</t>
   </si>
@@ -7283,6 +7283,9 @@
   </si>
   <si>
     <t xml:space="preserve">6008-2Z/C3 SKF BEARING – 8 euro cip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rulment </t>
   </si>
   <si>
     <t xml:space="preserve">11394-KUDU-E90</t>
@@ -7559,6 +7562,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -7649,10 +7653,18 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7661,50 +7673,52 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="24" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="7" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8033,7 +8047,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="5.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
@@ -35247,17 +35261,19 @@
       <c r="M683" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="N683" s="7"/>
+      <c r="N683" s="7" t="s">
+        <v>2421</v>
+      </c>
     </row>
     <row r="684" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A684" s="5" t="s">
-        <v>2421</v>
+        <v>2422</v>
       </c>
       <c r="B684" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C684" s="7" t="s">
-        <v>2422</v>
+        <v>2423</v>
       </c>
       <c r="D684" s="8"/>
       <c r="E684" s="7"/>
@@ -35266,7 +35282,7 @@
         <v>0.05</v>
       </c>
       <c r="H684" s="7" t="s">
-        <v>2423</v>
+        <v>2424</v>
       </c>
       <c r="I684" s="7" t="s">
         <v>36</v>
@@ -35287,13 +35303,13 @@
     </row>
     <row r="685" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A685" s="5" t="s">
-        <v>2424</v>
+        <v>2425</v>
       </c>
       <c r="B685" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C685" s="7" t="s">
-        <v>2425</v>
+        <v>2426</v>
       </c>
       <c r="D685" s="8"/>
       <c r="E685" s="7"/>
@@ -35302,7 +35318,7 @@
         <v>0.1</v>
       </c>
       <c r="H685" s="7" t="s">
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="I685" s="7" t="s">
         <v>262</v>
@@ -35318,18 +35334,18 @@
         <v>21</v>
       </c>
       <c r="N685" s="7" t="s">
-        <v>2427</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="686" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A686" s="5" t="s">
-        <v>2428</v>
+        <v>2429</v>
       </c>
       <c r="B686" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C686" s="7" t="s">
-        <v>2429</v>
+        <v>2430</v>
       </c>
       <c r="D686" s="8"/>
       <c r="E686" s="7"/>
@@ -35338,7 +35354,7 @@
         <v>0.05</v>
       </c>
       <c r="H686" s="7" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="I686" s="7" t="s">
         <v>36</v>
@@ -35359,13 +35375,13 @@
     </row>
     <row r="687" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A687" s="5" t="s">
-        <v>2431</v>
+        <v>2432</v>
       </c>
       <c r="B687" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C687" s="7" t="s">
-        <v>2432</v>
+        <v>2433</v>
       </c>
       <c r="D687" s="8"/>
       <c r="E687" s="7"/>
@@ -35374,7 +35390,7 @@
         <v>0.1</v>
       </c>
       <c r="H687" s="7" t="s">
-        <v>2433</v>
+        <v>2434</v>
       </c>
       <c r="I687" s="7" t="s">
         <v>851</v>
@@ -35395,13 +35411,13 @@
     </row>
     <row r="688" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A688" s="5" t="s">
-        <v>2434</v>
+        <v>2435</v>
       </c>
       <c r="B688" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C688" s="7" t="s">
-        <v>2435</v>
+        <v>2436</v>
       </c>
       <c r="D688" s="8"/>
       <c r="E688" s="7"/>
@@ -35410,7 +35426,7 @@
         <v>0.05</v>
       </c>
       <c r="H688" s="7" t="s">
-        <v>2436</v>
+        <v>2437</v>
       </c>
       <c r="I688" s="7" t="s">
         <v>17</v>
@@ -35426,18 +35442,18 @@
         <v>21</v>
       </c>
       <c r="N688" s="7" t="s">
-        <v>2437</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="689" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A689" s="5" t="s">
-        <v>2438</v>
+        <v>2439</v>
       </c>
       <c r="B689" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C689" s="7" t="s">
-        <v>2439</v>
+        <v>2440</v>
       </c>
       <c r="D689" s="8"/>
       <c r="E689" s="7"/>
@@ -35446,7 +35462,7 @@
         <v>0.05</v>
       </c>
       <c r="H689" s="7" t="s">
-        <v>2440</v>
+        <v>2441</v>
       </c>
       <c r="I689" s="7" t="s">
         <v>1811</v>
@@ -35462,18 +35478,18 @@
         <v>21</v>
       </c>
       <c r="N689" s="7" t="s">
-        <v>2441</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="690" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A690" s="5" t="s">
-        <v>2442</v>
+        <v>2443</v>
       </c>
       <c r="B690" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C690" s="7" t="s">
-        <v>2443</v>
+        <v>2444</v>
       </c>
       <c r="D690" s="8"/>
       <c r="E690" s="7"/>
@@ -35482,7 +35498,7 @@
         <v>0.15</v>
       </c>
       <c r="H690" s="7" t="s">
-        <v>2444</v>
+        <v>2445</v>
       </c>
       <c r="I690" s="7" t="s">
         <v>28</v>
@@ -35498,18 +35514,18 @@
         <v>21</v>
       </c>
       <c r="N690" s="7" t="s">
-        <v>2445</v>
+        <v>2446</v>
       </c>
     </row>
     <row r="691" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A691" s="5" t="s">
-        <v>2446</v>
+        <v>2447</v>
       </c>
       <c r="B691" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C691" s="7" t="s">
-        <v>2447</v>
+        <v>2448</v>
       </c>
       <c r="D691" s="8"/>
       <c r="E691" s="7"/>
@@ -35518,7 +35534,7 @@
         <v>2.5</v>
       </c>
       <c r="H691" s="7" t="s">
-        <v>2448</v>
+        <v>2449</v>
       </c>
       <c r="I691" s="7" t="s">
         <v>48</v>
@@ -35534,18 +35550,18 @@
         <v>21</v>
       </c>
       <c r="N691" s="7" t="s">
-        <v>2449</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="692" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A692" s="5" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="B692" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C692" s="7" t="s">
-        <v>2451</v>
+        <v>2452</v>
       </c>
       <c r="D692" s="8"/>
       <c r="E692" s="7"/>
@@ -35554,7 +35570,7 @@
         <v>2</v>
       </c>
       <c r="H692" s="7" t="s">
-        <v>2452</v>
+        <v>2453</v>
       </c>
       <c r="I692" s="7" t="s">
         <v>48</v>
@@ -35570,18 +35586,18 @@
         <v>21</v>
       </c>
       <c r="N692" s="7" t="s">
-        <v>2453</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="693" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A693" s="5" t="s">
-        <v>2454</v>
+        <v>2455</v>
       </c>
       <c r="B693" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C693" s="7" t="s">
-        <v>2455</v>
+        <v>2456</v>
       </c>
       <c r="D693" s="8"/>
       <c r="E693" s="7"/>
@@ -35590,7 +35606,7 @@
         <v>0.15</v>
       </c>
       <c r="H693" s="7" t="s">
-        <v>2456</v>
+        <v>2457</v>
       </c>
       <c r="I693" s="7" t="s">
         <v>1561</v>
@@ -35611,13 +35627,13 @@
     </row>
     <row r="694" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A694" s="5" t="s">
-        <v>2457</v>
+        <v>2458</v>
       </c>
       <c r="B694" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C694" s="7" t="s">
-        <v>2458</v>
+        <v>2459</v>
       </c>
       <c r="D694" s="8"/>
       <c r="E694" s="7"/>
@@ -35626,7 +35642,7 @@
         <v>0.05</v>
       </c>
       <c r="H694" s="7" t="s">
-        <v>2459</v>
+        <v>2460</v>
       </c>
       <c r="I694" s="7" t="s">
         <v>262</v>
@@ -35642,18 +35658,18 @@
         <v>21</v>
       </c>
       <c r="N694" s="7" t="s">
-        <v>2460</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="695" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A695" s="5" t="s">
-        <v>2461</v>
+        <v>2462</v>
       </c>
       <c r="B695" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C695" s="7" t="s">
-        <v>2462</v>
+        <v>2463</v>
       </c>
       <c r="D695" s="8"/>
       <c r="E695" s="7"/>
@@ -35662,7 +35678,7 @@
         <v>0.05</v>
       </c>
       <c r="H695" s="7" t="s">
-        <v>2463</v>
+        <v>2464</v>
       </c>
       <c r="I695" s="7" t="s">
         <v>1811</v>
@@ -35678,18 +35694,18 @@
         <v>21</v>
       </c>
       <c r="N695" s="7" t="s">
-        <v>2464</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="696" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A696" s="5" t="s">
-        <v>2465</v>
+        <v>2466</v>
       </c>
       <c r="B696" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C696" s="7" t="s">
-        <v>2466</v>
+        <v>2467</v>
       </c>
       <c r="D696" s="8"/>
       <c r="E696" s="7"/>
@@ -35698,7 +35714,7 @@
         <v>0.15</v>
       </c>
       <c r="H696" s="7" t="s">
-        <v>2467</v>
+        <v>2468</v>
       </c>
       <c r="I696" s="7" t="s">
         <v>776</v>
@@ -35714,18 +35730,18 @@
         <v>21</v>
       </c>
       <c r="N696" s="7" t="s">
-        <v>2468</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="697" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A697" s="5" t="s">
-        <v>2469</v>
+        <v>2470</v>
       </c>
       <c r="B697" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C697" s="7" t="s">
-        <v>2470</v>
+        <v>2471</v>
       </c>
       <c r="D697" s="8"/>
       <c r="E697" s="7"/>
@@ -35734,7 +35750,7 @@
         <v>0.05</v>
       </c>
       <c r="H697" s="7" t="s">
-        <v>2471</v>
+        <v>2472</v>
       </c>
       <c r="I697" s="7" t="s">
         <v>117</v>
@@ -35750,18 +35766,18 @@
         <v>21</v>
       </c>
       <c r="N697" s="7" t="s">
-        <v>2472</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="698" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A698" s="5" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="B698" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C698" s="7" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="D698" s="8"/>
       <c r="E698" s="7"/>
@@ -35770,7 +35786,7 @@
         <v>0.05</v>
       </c>
       <c r="H698" s="7" t="s">
-        <v>2475</v>
+        <v>2476</v>
       </c>
       <c r="I698" s="7" t="s">
         <v>117</v>
@@ -35786,18 +35802,18 @@
         <v>21</v>
       </c>
       <c r="N698" s="7" t="s">
-        <v>2472</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="699" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A699" s="5" t="s">
-        <v>2476</v>
+        <v>2477</v>
       </c>
       <c r="B699" s="6" t="n">
         <v>4</v>
       </c>
       <c r="C699" s="7" t="s">
-        <v>2477</v>
+        <v>2478</v>
       </c>
       <c r="D699" s="8"/>
       <c r="E699" s="7"/>
@@ -35806,7 +35822,7 @@
         <v>0.03</v>
       </c>
       <c r="H699" s="7" t="s">
-        <v>2478</v>
+        <v>2479</v>
       </c>
       <c r="I699" s="7" t="s">
         <v>206</v>
@@ -35822,18 +35838,18 @@
         <v>21</v>
       </c>
       <c r="N699" s="7" t="s">
-        <v>2479</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="700" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A700" s="5" t="s">
-        <v>2480</v>
+        <v>2481</v>
       </c>
       <c r="B700" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C700" s="7" t="s">
-        <v>2481</v>
+        <v>2482</v>
       </c>
       <c r="D700" s="8"/>
       <c r="E700" s="7"/>
@@ -35842,7 +35858,7 @@
         <v>0.15</v>
       </c>
       <c r="H700" s="7" t="s">
-        <v>2482</v>
+        <v>2483</v>
       </c>
       <c r="I700" s="7" t="s">
         <v>262</v>
@@ -35858,18 +35874,18 @@
         <v>21</v>
       </c>
       <c r="N700" s="7" t="s">
-        <v>2483</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="701" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A701" s="5" t="s">
-        <v>2484</v>
+        <v>2485</v>
       </c>
       <c r="B701" s="6" t="n">
         <v>1</v>
       </c>
       <c r="C701" s="7" t="s">
-        <v>2485</v>
+        <v>2486</v>
       </c>
       <c r="D701" s="8"/>
       <c r="E701" s="7"/>
@@ -35878,7 +35894,7 @@
         <v>0.1</v>
       </c>
       <c r="H701" s="7" t="s">
-        <v>2486</v>
+        <v>2487</v>
       </c>
       <c r="I701" s="7" t="s">
         <v>624</v>
@@ -35899,19 +35915,19 @@
     </row>
     <row r="702" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A702" s="1" t="s">
-        <v>2487</v>
+        <v>2488</v>
       </c>
       <c r="B702" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C702" s="1" t="s">
-        <v>2488</v>
+        <v>2489</v>
       </c>
       <c r="G702" s="1" t="n">
         <v>0.05</v>
       </c>
       <c r="H702" s="1" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
       <c r="I702" s="7" t="s">
         <v>262</v>
@@ -35927,24 +35943,24 @@
         <v>21</v>
       </c>
       <c r="N702" s="1" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="703" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A703" s="1" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
       <c r="B703" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C703" s="1" t="s">
-        <v>2492</v>
+        <v>2493</v>
       </c>
       <c r="G703" s="1" t="n">
         <v>0.1</v>
       </c>
       <c r="H703" s="1" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
       <c r="I703" s="1" t="s">
         <v>1341</v>
@@ -35965,19 +35981,19 @@
     </row>
     <row r="704" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A704" s="1" t="s">
-        <v>2494</v>
+        <v>2495</v>
       </c>
       <c r="B704" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C704" s="1" t="s">
-        <v>2495</v>
+        <v>2496</v>
       </c>
       <c r="G704" s="1" t="n">
         <v>0.15</v>
       </c>
       <c r="H704" s="1" t="s">
-        <v>2496</v>
+        <v>2497</v>
       </c>
       <c r="I704" s="1" t="s">
         <v>117</v>
@@ -35993,24 +36009,24 @@
         <v>21</v>
       </c>
       <c r="N704" s="1" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="705" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A705" s="1" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="B705" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C705" s="1" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="G705" s="1" t="n">
         <v>0.2</v>
       </c>
       <c r="H705" s="1" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="I705" s="1" t="s">
         <v>1085</v>
@@ -36026,24 +36042,24 @@
         <v>21</v>
       </c>
       <c r="N705" s="1" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="706" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A706" s="1" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="B706" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C706" s="1" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
       <c r="G706" s="1" t="n">
         <v>0.5</v>
       </c>
       <c r="H706" s="1" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="I706" s="1" t="s">
         <v>206</v>
@@ -36059,7 +36075,7 @@
         <v>21</v>
       </c>
       <c r="N706" s="1" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="707" customFormat="false" ht="13.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>